<commit_message>
Fix XLSX template: single sheet, gray example text, no background color
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KoEmo_template.xlsx
+++ b/docs/KoEmo_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -42,12 +46,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
         <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E2F3"/>
-        <bgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +72,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -585,114 +583,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>감정 표현</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>긍정 감정</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>기쁘다, 반갑다, 흐뭇하다, 뿌듯하다</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>흐뭇했다</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>아들이 독립한 뒤 처음으로 월급을 타서 부모님께 선물을 사왔다. 선물을 받아든 어머니의 마음이 ___.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>감정 표현</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>긍정 감정</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>기쁘다, 반갑다, 흐뭇하다, 뿌듯하다</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>뿌듯했다</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>6개월간 준비한 자격증 시험에 합격했다는 문자를 받았다. 그동안의 노력이 보상받는 느낌이라 ___.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>감정 표현</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>긍정 감정</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>기쁘다, 반갑다, 흐뭇하다, 뿌듯하다</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>반가웠다</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>오랜만에 연락 없던 고향 친구에게서 전화가 왔다. 목소리를 들으니 정말 ___.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>감정 표현</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>긍정 감정</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>기쁘다, 반갑다, 흐뭇하다, 뿌듯하다</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>기뻤다</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>복권에 당첨되었다는 소식을 듣고 어찌할 바를 몰라 너무 ___.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 번호 column to template, mark examples as (예시)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KoEmo_template.xlsx
+++ b/docs/KoEmo_template.xlsx
@@ -438,38 +438,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>도메인</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>단어군</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>정답</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상황</t>
         </is>
@@ -478,25 +484,30 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>(예시)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>감각 표현</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>미각</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>맵다, 얼큰하다, 알싸하다, 칼칼하다</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>얼큰하다</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>추운 겨울날 순대국밥 국물을 한 숟갈 떠먹으니 속이 확 풀리는 것이 국물이 참 ___.</t>
         </is>
@@ -505,25 +516,30 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>(예시)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>감각 표현</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>미각</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>맵다, 얼큰하다, 알싸하다, 칼칼하다</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>알싸하다</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>초밥 위 와사비를 너무 많이 찍어 먹었더니 코끝이 찡하고 눈물이 핑 돌았다. 와사비가 ___.</t>
         </is>
@@ -532,25 +548,30 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>(예시)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>감각 표현</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>미각</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>맵다, 얼큰하다, 알싸하다, 칼칼하다</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>맵다</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>라면에 고춧가루를 잔뜩 넣었더니 그냥 ___ 먹기 힘들었다.</t>
         </is>
@@ -559,25 +580,30 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>(예시)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
           <t>감각 표현</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>미각</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>맵다, 얼큰하다, 알싸하다, 칼칼하다</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>칼칼하다</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>김치찌개에 청양고추를 넣었더니 국물 넘길 때 목구멍이 얼얼하게 ___.</t>
         </is>

</xml_diff>

<commit_message>
Add domain dropdown to XLSX template
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KoEmo_template.xlsx
+++ b/docs/KoEmo_template.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="620" windowWidth="51200" windowHeight="28180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="KoEmo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,12 +25,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00666666"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF666666"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -44,8 +47,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,24 +61,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -438,12 +460,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F105"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" style="6" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
@@ -482,7 +503,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>(예시)</t>
         </is>
@@ -514,7 +535,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>(예시)</t>
         </is>
@@ -546,7 +567,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>(예시)</t>
         </is>
@@ -573,12 +594,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>라면에 고춧가루를 잔뜩 넣었더니 그냥 ___ 먹기 힘들었다.</t>
+          <t>라면에 고춧가루를 잔뜩 넣었더니 그냥 먹기 힘들게 ___.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>(예시)</t>
         </is>
@@ -605,11 +626,1016 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>김치찌개에 청양고추를 넣었더니 국물 넘길 때 목구멍이 얼얼하게 ___.</t>
-        </is>
-      </c>
+          <t>김치찌개에 청양고추를 넣었더니 국물 넘길 때 목구멍이 ___.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="3" t="n"/>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="3" t="n"/>
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="3" t="n"/>
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="3" t="n"/>
+      <c r="E47" s="3" t="n"/>
+      <c r="F47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="3" t="n"/>
+      <c r="D48" s="3" t="n"/>
+      <c r="E48" s="3" t="n"/>
+      <c r="F48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="3" t="n"/>
+      <c r="D49" s="3" t="n"/>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="3" t="n"/>
+      <c r="C50" s="3" t="n"/>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="3" t="n"/>
+      <c r="F50" s="3" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="3" t="n"/>
+      <c r="C51" s="3" t="n"/>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="3" t="n"/>
+      <c r="C52" s="3" t="n"/>
+      <c r="D52" s="3" t="n"/>
+      <c r="E52" s="3" t="n"/>
+      <c r="F52" s="3" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="3" t="n"/>
+      <c r="C53" s="3" t="n"/>
+      <c r="D53" s="3" t="n"/>
+      <c r="E53" s="3" t="n"/>
+      <c r="F53" s="3" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="3" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" s="3" t="n"/>
+      <c r="C55" s="3" t="n"/>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="n"/>
+      <c r="F55" s="3" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" s="3" t="n"/>
+      <c r="C56" s="3" t="n"/>
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="3" t="n"/>
+      <c r="F56" s="3" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B57" s="3" t="n"/>
+      <c r="C57" s="3" t="n"/>
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="3" t="n"/>
+      <c r="F57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="B58" s="3" t="n"/>
+      <c r="C58" s="3" t="n"/>
+      <c r="D58" s="3" t="n"/>
+      <c r="E58" s="3" t="n"/>
+      <c r="F58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B59" s="3" t="n"/>
+      <c r="C59" s="3" t="n"/>
+      <c r="D59" s="3" t="n"/>
+      <c r="E59" s="3" t="n"/>
+      <c r="F59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="B60" s="3" t="n"/>
+      <c r="C60" s="3" t="n"/>
+      <c r="D60" s="3" t="n"/>
+      <c r="E60" s="3" t="n"/>
+      <c r="F60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B61" s="3" t="n"/>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="B62" s="3" t="n"/>
+      <c r="C62" s="3" t="n"/>
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="3" t="n"/>
+      <c r="F62" s="3" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B63" s="3" t="n"/>
+      <c r="C63" s="3" t="n"/>
+      <c r="D63" s="3" t="n"/>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="B64" s="3" t="n"/>
+      <c r="C64" s="3" t="n"/>
+      <c r="D64" s="3" t="n"/>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B65" s="3" t="n"/>
+      <c r="C65" s="3" t="n"/>
+      <c r="D65" s="3" t="n"/>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="3" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="3" t="n"/>
+      <c r="D69" s="3" t="n"/>
+      <c r="E69" s="3" t="n"/>
+      <c r="F69" s="3" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="B70" s="3" t="n"/>
+      <c r="C70" s="3" t="n"/>
+      <c r="D70" s="3" t="n"/>
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="3" t="n"/>
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="3" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="B72" s="3" t="n"/>
+      <c r="C72" s="3" t="n"/>
+      <c r="D72" s="3" t="n"/>
+      <c r="E72" s="3" t="n"/>
+      <c r="F72" s="3" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="3" t="n"/>
+      <c r="D73" s="3" t="n"/>
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="B74" s="3" t="n"/>
+      <c r="C74" s="3" t="n"/>
+      <c r="D74" s="3" t="n"/>
+      <c r="E74" s="3" t="n"/>
+      <c r="F74" s="3" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B75" s="3" t="n"/>
+      <c r="C75" s="3" t="n"/>
+      <c r="D75" s="3" t="n"/>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" s="3" t="n"/>
+      <c r="C76" s="3" t="n"/>
+      <c r="D76" s="3" t="n"/>
+      <c r="E76" s="3" t="n"/>
+      <c r="F76" s="3" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="B77" s="3" t="n"/>
+      <c r="C77" s="3" t="n"/>
+      <c r="D77" s="3" t="n"/>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="B78" s="3" t="n"/>
+      <c r="C78" s="3" t="n"/>
+      <c r="D78" s="3" t="n"/>
+      <c r="E78" s="3" t="n"/>
+      <c r="F78" s="3" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B79" s="3" t="n"/>
+      <c r="C79" s="3" t="n"/>
+      <c r="D79" s="3" t="n"/>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="3" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="B80" s="3" t="n"/>
+      <c r="C80" s="3" t="n"/>
+      <c r="D80" s="3" t="n"/>
+      <c r="E80" s="3" t="n"/>
+      <c r="F80" s="3" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B81" s="3" t="n"/>
+      <c r="C81" s="3" t="n"/>
+      <c r="D81" s="3" t="n"/>
+      <c r="E81" s="3" t="n"/>
+      <c r="F81" s="3" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="B82" s="3" t="n"/>
+      <c r="C82" s="3" t="n"/>
+      <c r="D82" s="3" t="n"/>
+      <c r="E82" s="3" t="n"/>
+      <c r="F82" s="3" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="B83" s="3" t="n"/>
+      <c r="C83" s="3" t="n"/>
+      <c r="D83" s="3" t="n"/>
+      <c r="E83" s="3" t="n"/>
+      <c r="F83" s="3" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="B84" s="3" t="n"/>
+      <c r="C84" s="3" t="n"/>
+      <c r="D84" s="3" t="n"/>
+      <c r="E84" s="3" t="n"/>
+      <c r="F84" s="3" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="3" t="n"/>
+      <c r="D85" s="3" t="n"/>
+      <c r="E85" s="3" t="n"/>
+      <c r="F85" s="3" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="3" t="n"/>
+      <c r="D86" s="3" t="n"/>
+      <c r="E86" s="3" t="n"/>
+      <c r="F86" s="3" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="B87" s="3" t="n"/>
+      <c r="C87" s="3" t="n"/>
+      <c r="D87" s="3" t="n"/>
+      <c r="E87" s="3" t="n"/>
+      <c r="F87" s="3" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="B88" s="3" t="n"/>
+      <c r="C88" s="3" t="n"/>
+      <c r="D88" s="3" t="n"/>
+      <c r="E88" s="3" t="n"/>
+      <c r="F88" s="3" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="3" t="n"/>
+      <c r="D89" s="3" t="n"/>
+      <c r="E89" s="3" t="n"/>
+      <c r="F89" s="3" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="3" t="n"/>
+      <c r="D90" s="3" t="n"/>
+      <c r="E90" s="3" t="n"/>
+      <c r="F90" s="3" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="B91" s="3" t="n"/>
+      <c r="C91" s="3" t="n"/>
+      <c r="D91" s="3" t="n"/>
+      <c r="E91" s="3" t="n"/>
+      <c r="F91" s="3" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="B92" s="3" t="n"/>
+      <c r="C92" s="3" t="n"/>
+      <c r="D92" s="3" t="n"/>
+      <c r="E92" s="3" t="n"/>
+      <c r="F92" s="3" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="3" t="n"/>
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="3" t="n"/>
+      <c r="F93" s="3" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="3" t="n"/>
+      <c r="D94" s="3" t="n"/>
+      <c r="E94" s="3" t="n"/>
+      <c r="F94" s="3" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="3" t="n"/>
+      <c r="D95" s="3" t="n"/>
+      <c r="E95" s="3" t="n"/>
+      <c r="F95" s="3" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="B96" s="3" t="n"/>
+      <c r="C96" s="3" t="n"/>
+      <c r="D96" s="3" t="n"/>
+      <c r="E96" s="3" t="n"/>
+      <c r="F96" s="3" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="3" t="n"/>
+      <c r="D97" s="3" t="n"/>
+      <c r="E97" s="3" t="n"/>
+      <c r="F97" s="3" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="3" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="3" t="n"/>
+      <c r="D99" s="3" t="n"/>
+      <c r="E99" s="3" t="n"/>
+      <c r="F99" s="3" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="B100" s="3" t="n"/>
+      <c r="C100" s="3" t="n"/>
+      <c r="D100" s="3" t="n"/>
+      <c r="E100" s="3" t="n"/>
+      <c r="F100" s="3" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="B101" s="3" t="n"/>
+      <c r="C101" s="3" t="n"/>
+      <c r="D101" s="3" t="n"/>
+      <c r="E101" s="3" t="n"/>
+      <c r="F101" s="3" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="n">
+        <v>97</v>
+      </c>
+      <c r="B102" s="3" t="n"/>
+      <c r="C102" s="3" t="n"/>
+      <c r="D102" s="3" t="n"/>
+      <c r="E102" s="3" t="n"/>
+      <c r="F102" s="3" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="n">
+        <v>98</v>
+      </c>
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
+      <c r="D103" s="3" t="n"/>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="3" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="B104" s="3" t="n"/>
+      <c r="C104" s="3" t="n"/>
+      <c r="D104" s="3" t="n"/>
+      <c r="E104" s="3" t="n"/>
+      <c r="F104" s="3" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B105" s="3" t="n"/>
+      <c r="C105" s="3" t="n"/>
+      <c r="D105" s="3" t="n"/>
+      <c r="E105" s="3" t="n"/>
+      <c r="F105" s="3" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B6:B105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="도메인 선택 오류" error="5가지 도메인 중에서 선택해 주세요." promptTitle="도메인" prompt="도메인을 선택하세요." type="list">
+      <formula1>"감각 표현,감정 표현,판단 표현,감상 표현,상징 표현"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>